<commit_message>
Fix chart legend and category axis parity
</commit_message>
<xml_diff>
--- a/tests/fixtures/charts/line-pie-area-scatter.xlsx
+++ b/tests/fixtures/charts/line-pie-area-scatter.xlsx
@@ -321,15 +321,15 @@
             <c:spPr/>
           </c:marker>
         </c:ser>
-        <c:axId val="61662731"/>
-        <c:axId val="40152173"/>
+        <c:axId val="54091649"/>
+        <c:axId val="86126836"/>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:smooth val="0"/>
         <c:marker val="0"/>
       </c:lineChart>
       <c:catAx axisType="0">
-        <c:axId val="61662731"/>
+        <c:axId val="54091649"/>
         <c:delete val="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -383,10 +383,10 @@
         <c:tickMarkSkip val="1"/>
         <c:noMultiLvlLbl val="1"/>
         <c:crosses val="autoZero"/>
-        <c:crossAx val="40152173"/>
+        <c:crossAx val="86126836"/>
       </c:catAx>
       <c:valAx axisType="3">
-        <c:axId val="40152173"/>
+        <c:axId val="86126836"/>
         <c:delete val="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -446,7 +446,7 @@
         </c:majorGridlines>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
-        <c:crossAx val="61662731"/>
+        <c:crossAx val="54091649"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -714,13 +714,13 @@
           </c:val>
           <c:extLst/>
         </c:ser>
-        <c:axId val="69991686"/>
-        <c:axId val="81927213"/>
+        <c:axId val="54051826"/>
+        <c:axId val="37735241"/>
         <c:varyColors val="0"/>
         <c:grouping val="stacked"/>
       </c:areaChart>
       <c:catAx axisType="0">
-        <c:axId val="69991686"/>
+        <c:axId val="54051826"/>
         <c:delete val="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -774,10 +774,10 @@
         <c:tickMarkSkip val="1"/>
         <c:noMultiLvlLbl val="1"/>
         <c:crosses val="autoZero"/>
-        <c:crossAx val="81927213"/>
+        <c:crossAx val="37735241"/>
       </c:catAx>
       <c:valAx axisType="3">
-        <c:axId val="81927213"/>
+        <c:axId val="37735241"/>
         <c:delete val="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -837,7 +837,7 @@
         </c:majorGridlines>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
-        <c:crossAx val="69991686"/>
+        <c:crossAx val="54051826"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -1216,13 +1216,13 @@
             <c:spPr/>
           </c:marker>
         </c:ser>
-        <c:axId val="12571534"/>
-        <c:axId val="53749282"/>
+        <c:axId val="34483659"/>
+        <c:axId val="91258079"/>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
       </c:scatterChart>
       <c:valAx axisType="3">
-        <c:axId val="12571534"/>
+        <c:axId val="34483659"/>
         <c:delete val="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1272,10 +1272,10 @@
           </a:p>
         </c:txPr>
         <c:crosses val="autoZero"/>
-        <c:crossAx val="53749282"/>
+        <c:crossAx val="91258079"/>
       </c:valAx>
       <c:valAx axisType="3">
-        <c:axId val="53749282"/>
+        <c:axId val="91258079"/>
         <c:delete val="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1335,7 +1335,7 @@
         </c:majorGridlines>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
-        <c:crossAx val="12571534"/>
+        <c:crossAx val="34483659"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -4617,7 +4617,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{072B6BD8-3558-B9C8-AAB8-C79677E7FE08}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{014053F4-9248-47B8-1258-1237AC434FC8}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
   <sheetData>

</xml_diff>